<commit_message>
examples updated + gl well from pwf button
</commit_message>
<xml_diff>
--- a/examples/ex051.MF_pipeline.xlsx
+++ b/examples/ex051.MF_pipeline.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr codeName="ЭтаКнига"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <workbookPr codeName="ЭтаКнига" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\unifloc_vba\examples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\unifloc\unifloc_vba\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BD17EC-C962-474D-9CA3-00171A5EEC8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="-20820" windowWidth="31530" windowHeight="19905"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{4F3269D6-54F3-4796-9400-98B76DA490E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -18,13 +19,14 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="feed_json">Лист1!$I$58</definedName>
-    <definedName name="pipe_construction">Лист1!$Q$4</definedName>
-    <definedName name="pipe_object">Лист1!$S$31</definedName>
-    <definedName name="PVT_json">Лист1!$I$53</definedName>
-    <definedName name="t_model">Лист1!$Q$13</definedName>
+    <definedName name="feed_json">Лист1!$D$17</definedName>
+    <definedName name="pipe_diam">Лист1!$K$3</definedName>
+    <definedName name="pipe_object">Лист1!$D$35</definedName>
+    <definedName name="pipe_trajectory">Лист1!$H$3</definedName>
+    <definedName name="PVT_json">Лист1!$D$12</definedName>
+    <definedName name="t_model">Лист1!$N$16</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,6 +38,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -43,24 +47,114 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
+  <si>
+    <t>gamma_gas</t>
+  </si>
+  <si>
+    <t>gamma_oil</t>
+  </si>
+  <si>
+    <t>gamma_wat</t>
+  </si>
+  <si>
+    <t>rsb_m3m3</t>
+  </si>
+  <si>
+    <t>pb_atma</t>
+  </si>
+  <si>
+    <t>t_res_C</t>
+  </si>
+  <si>
+    <t>bob_m3m3</t>
+  </si>
+  <si>
+    <t>muob_cP</t>
+  </si>
+  <si>
+    <t>pvt_corr_set</t>
+  </si>
+  <si>
+    <t>PVT</t>
+  </si>
+  <si>
+    <t>q_liq_sm3day</t>
+  </si>
+  <si>
+    <t>fw_perc</t>
+  </si>
+  <si>
+    <t>rp_m3m3</t>
+  </si>
+  <si>
+    <t>q_gas_free_sm3day</t>
+  </si>
+  <si>
+    <t>feed</t>
+  </si>
   <si>
     <t>trajectory</t>
   </si>
   <si>
+    <t>hmes, m</t>
+  </si>
+  <si>
+    <t>hvert, m</t>
+  </si>
+  <si>
+    <t>roughness_m</t>
+  </si>
+  <si>
     <t>diameter</t>
   </si>
   <si>
-    <t>hmes, m</t>
-  </si>
-  <si>
-    <t>hvert, m</t>
-  </si>
-  <si>
     <t>diam, mm</t>
   </si>
   <si>
-    <t>construction</t>
+    <t>pipe diams</t>
+  </si>
+  <si>
+    <t>t model</t>
+  </si>
+  <si>
+    <t>t_start_C</t>
+  </si>
+  <si>
+    <t>t_end_C</t>
+  </si>
+  <si>
+    <t>thermal_conductivity_formation_WmC</t>
+  </si>
+  <si>
+    <t>specific_heat_capacity_formation_JkgC</t>
+  </si>
+  <si>
+    <t>thermal_conductivity_cement_WmC</t>
+  </si>
+  <si>
+    <t>thermal_conductivity_tubing_WmC</t>
+  </si>
+  <si>
+    <t>thermal_conductivity_casing_WmC</t>
+  </si>
+  <si>
+    <t>heat_transfer_casing_liquid_Wm2C</t>
+  </si>
+  <si>
+    <t>heat_transfer_casing_gas_Wm2C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heat_transfer_fluid_convection_Wm2C </t>
+  </si>
+  <si>
+    <t>time_calc_hr</t>
+  </si>
+  <si>
+    <t>param</t>
+  </si>
+  <si>
+    <t>json</t>
   </si>
   <si>
     <t>ambient temperature</t>
@@ -69,7 +163,7 @@
     <t>t amb, C</t>
   </si>
   <si>
-    <t>t model</t>
+    <t>diam</t>
   </si>
   <si>
     <t>t_model</t>
@@ -108,90 +202,27 @@
     <t>pipe_object</t>
   </si>
   <si>
-    <t>feed</t>
-  </si>
-  <si>
     <t>calc_along_coord</t>
   </si>
   <si>
-    <t>param</t>
-  </si>
-  <si>
     <t>{"show_array":1}</t>
-  </si>
-  <si>
-    <t>q_liq_sm3day</t>
-  </si>
-  <si>
-    <t>fw_perc</t>
-  </si>
-  <si>
-    <t>rp_m3m3</t>
-  </si>
-  <si>
-    <t>q_gas_free_sm3day</t>
-  </si>
-  <si>
-    <t>4 шага для построения кривой распределения давления в вертикальной трубе</t>
-  </si>
-  <si>
-    <t>1. Задать конструкцию/инклинометрию и диаметры</t>
-  </si>
-  <si>
-    <t>2. Задать температурную модель</t>
-  </si>
-  <si>
-    <t>3. Задать объект для трубы - включает ссылки на конструкцию и температурную модель</t>
-  </si>
-  <si>
-    <t>4. Запустить пример расчета распределения давления и температуры в трубе</t>
-  </si>
-  <si>
-    <t>gamma_gas</t>
-  </si>
-  <si>
-    <t>gamma_oil</t>
-  </si>
-  <si>
-    <t>gamma_wat</t>
-  </si>
-  <si>
-    <t>rsb_m3m3</t>
-  </si>
-  <si>
-    <t>pb_atma</t>
-  </si>
-  <si>
-    <t>t_res_C</t>
-  </si>
-  <si>
-    <t>bob_m3m3</t>
-  </si>
-  <si>
-    <t>muob_cP</t>
-  </si>
-  <si>
-    <t>pvt_corr_set</t>
-  </si>
-  <si>
-    <t>PVT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -213,12 +244,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA0FAFA"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6FA64"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -252,9 +277,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -289,7 +314,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -357,76 +381,76 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Лист1!$T$47:$T$66</c:f>
+              <c:f>Лист1!$L$38:$L$57</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
-                  <c:v>10</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24.836360057558057</c:v>
+                  <c:v>37.211265919476702</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>39.660912169855287</c:v>
+                  <c:v>49.336935976810224</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>54.473728023011631</c:v>
+                  <c:v>61.368662604850357</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>69.274877304399666</c:v>
+                  <c:v>66.154734668379703</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>84.064262054326051</c:v>
+                  <c:v>73.301276031794316</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>98.841955005012849</c:v>
+                  <c:v>85.131937480979204</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>113.60819486374973</c:v>
+                  <c:v>96.859528861433972</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>128.36305394047776</c:v>
+                  <c:v>108.25265963744981</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>143.10660666796306</c:v>
+                  <c:v>118.64374732377269</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>157.83860705561924</c:v>
+                  <c:v>129.01643292775486</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>172.55946291726846</c:v>
+                  <c:v>139.37296783267652</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>187.26925720901431</c:v>
+                  <c:v>149.71212069474134</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>201.96807608679808</c:v>
+                  <c:v>160.03289583994723</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>216.65585276159905</c:v>
+                  <c:v>170.33447407582048</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>231.33268489206455</c:v>
+                  <c:v>180.15967523685279</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>233.09334496046432</c:v>
+                  <c:v>182.71586855800516</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>245.98725456824823</c:v>
+                  <c:v>189.28532313169057</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>260.62969555631469</c:v>
+                  <c:v>198.40957045644666</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>275.2616896761848</c:v>
+                  <c:v>207.53360232980467</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Лист1!$R$47:$R$66</c:f>
+              <c:f>Лист1!$J$38:$J$57</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="20"/>
@@ -434,58 +458,58 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>138.88888888888889</c:v>
+                  <c:v>147.05882352941177</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>277.77777777777777</c:v>
+                  <c:v>294.11764705882354</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>416.66666666666663</c:v>
+                  <c:v>441.1764705882353</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>555.55555555555554</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>694.44444444444446</c:v>
+                  <c:v>588.23529411764707</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>833.33333333333326</c:v>
+                  <c:v>735.29411764705878</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>972.22222222222217</c:v>
+                  <c:v>882.35294117647061</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1111.1111111111111</c:v>
+                  <c:v>1029.4117647058824</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1250</c:v>
+                  <c:v>1176.4705882352941</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1388.8888888888889</c:v>
+                  <c:v>1323.5294117647059</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1527.7777777777778</c:v>
+                  <c:v>1470.5882352941176</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1666.6666666666665</c:v>
+                  <c:v>1617.6470588235295</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1805.5555555555554</c:v>
+                  <c:v>1764.7058823529412</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1944.4444444444443</c:v>
+                  <c:v>1911.7647058823529</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2083.3333333333335</c:v>
+                  <c:v>2058.8235294117649</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>2100</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2222.2222222222222</c:v>
+                  <c:v>2205.8823529411766</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2361.1111111111109</c:v>
+                  <c:v>2352.9411764705883</c:v>
                 </c:pt>
                 <c:pt idx="19">
                   <c:v>2500</c:v>
@@ -496,7 +520,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000007-7E77-448C-89FD-68EFD1E409E3}"/>
+              <c16:uniqueId val="{00000007-5CBF-4CA0-AF72-B4A80B7F89FD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -508,11 +532,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="711548288"/>
-        <c:axId val="1204215664"/>
+        <c:axId val="1235903023"/>
+        <c:axId val="1235887183"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="711548288"/>
+        <c:axId val="1235903023"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -558,7 +582,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -625,12 +648,12 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1204215664"/>
+        <c:crossAx val="1235887183"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1204215664"/>
+        <c:axId val="1235887183"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -676,7 +699,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -743,7 +765,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="711548288"/>
+        <c:crossAx val="1235903023"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -757,7 +779,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -789,7 +810,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -797,6 +817,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -871,7 +892,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -939,7 +959,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Лист1!$U$47:$U$66</c:f>
+              <c:f>Лист1!$M$38:$M$57</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="20"/>
@@ -947,68 +967,68 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.666666666666666</c:v>
+                  <c:v>13.676470588235293</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15.333333333333334</c:v>
+                  <c:v>17.352941176470587</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18</c:v>
+                  <c:v>21.029411764705884</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20.666666666666664</c:v>
+                  <c:v>22.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>23.333333333333332</c:v>
+                  <c:v>24.705882352941178</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>26</c:v>
+                  <c:v>28.382352941176471</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>28.666666666666664</c:v>
+                  <c:v>32.058823529411768</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>31.333333333333332</c:v>
+                  <c:v>36.191176470588239</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>34</c:v>
+                  <c:v>42.147058823529413</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36.666666666666664</c:v>
+                  <c:v>48.102941176470587</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>39.333333333333329</c:v>
+                  <c:v>54.058823529411761</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>41.999999999999993</c:v>
+                  <c:v>60.014705882352942</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>44.666666666666657</c:v>
+                  <c:v>65.970588235294116</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>47.333333333333329</c:v>
+                  <c:v>71.92647058823529</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>50</c:v>
+                  <c:v>77.617647058823536</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>50.319999999999993</c:v>
+                  <c:v>79.099999999999994</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>52.666666666666664</c:v>
+                  <c:v>81.294117647058826</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>55.333333333333329</c:v>
+                  <c:v>83.647058823529406</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>57.999999999999993</c:v>
+                  <c:v>86</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Лист1!$S$47:$S$66</c:f>
+              <c:f>Лист1!$K$38:$K$57</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1016,61 +1036,61 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>138.88888888888889</c:v>
+                  <c:v>147.05882352941177</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>277.77777777777777</c:v>
+                  <c:v>294.11764705882354</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>416.66666666666663</c:v>
+                  <c:v>441.1764705882353</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>555.55555555555554</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>694.44444444444446</c:v>
+                  <c:v>588.23529411764707</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>833.33333333333326</c:v>
+                  <c:v>735.29411764705878</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>972.22222222222217</c:v>
+                  <c:v>882.35294117647061</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1111.1111111111111</c:v>
+                  <c:v>1026.4705882352941</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1250</c:v>
+                  <c:v>1158.8235294117646</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1388.8888888888889</c:v>
+                  <c:v>1291.1764705882354</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1527.7777777777778</c:v>
+                  <c:v>1423.5294117647059</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1666.6666666666665</c:v>
+                  <c:v>1555.8823529411766</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1805.5555555555554</c:v>
+                  <c:v>1688.2352941176471</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1944.4444444444443</c:v>
+                  <c:v>1820.5882352941176</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2083.3333333333335</c:v>
+                  <c:v>1947.0588235294119</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2100</c:v>
+                  <c:v>1980</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2222.2222222222222</c:v>
+                  <c:v>2064.7058823529414</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2361.1111111111109</c:v>
+                  <c:v>2182.3529411764707</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2500</c:v>
+                  <c:v>2300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1078,7 +1098,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000007-8E52-4609-B15F-ADFD5A2DC54B}"/>
+              <c16:uniqueId val="{00000007-AEB0-4BDA-973B-92593FC7D8B6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1114,7 +1134,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Лист1!$V$47:$V$66</c:f>
+              <c:f>Лист1!$N$38:$N$57</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1122,68 +1142,68 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.666666666666666</c:v>
+                  <c:v>13.676470588235293</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15.333333333333334</c:v>
+                  <c:v>17.352941176470587</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18</c:v>
+                  <c:v>21.029411764705884</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20.666666666666664</c:v>
+                  <c:v>22.5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>23.333333333333332</c:v>
+                  <c:v>24.705882352941178</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>26</c:v>
+                  <c:v>28.382352941176471</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>28.666666666666664</c:v>
+                  <c:v>32.058823529411768</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>31.333333333333332</c:v>
+                  <c:v>36.191176470588239</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>34</c:v>
+                  <c:v>42.147058823529413</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36.666666666666664</c:v>
+                  <c:v>48.102941176470587</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>39.333333333333329</c:v>
+                  <c:v>54.058823529411761</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>41.999999999999993</c:v>
+                  <c:v>60.014705882352942</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>44.666666666666657</c:v>
+                  <c:v>65.970588235294116</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>47.333333333333329</c:v>
+                  <c:v>71.92647058823529</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>50</c:v>
+                  <c:v>77.617647058823536</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>50.319999999999993</c:v>
+                  <c:v>79.099999999999994</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>52.666666666666664</c:v>
+                  <c:v>81.294117647058826</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>55.333333333333329</c:v>
+                  <c:v>83.647058823529406</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>57.999999999999993</c:v>
+                  <c:v>86</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Лист1!$S$47:$S$66</c:f>
+              <c:f>Лист1!$K$38:$K$57</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1191,61 +1211,61 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>138.88888888888889</c:v>
+                  <c:v>147.05882352941177</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>277.77777777777777</c:v>
+                  <c:v>294.11764705882354</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>416.66666666666663</c:v>
+                  <c:v>441.1764705882353</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>555.55555555555554</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>694.44444444444446</c:v>
+                  <c:v>588.23529411764707</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>833.33333333333326</c:v>
+                  <c:v>735.29411764705878</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>972.22222222222217</c:v>
+                  <c:v>882.35294117647061</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1111.1111111111111</c:v>
+                  <c:v>1026.4705882352941</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1250</c:v>
+                  <c:v>1158.8235294117646</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1388.8888888888889</c:v>
+                  <c:v>1291.1764705882354</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1527.7777777777778</c:v>
+                  <c:v>1423.5294117647059</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1666.6666666666665</c:v>
+                  <c:v>1555.8823529411766</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1805.5555555555554</c:v>
+                  <c:v>1688.2352941176471</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1944.4444444444443</c:v>
+                  <c:v>1820.5882352941176</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2083.3333333333335</c:v>
+                  <c:v>1947.0588235294119</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2100</c:v>
+                  <c:v>1980</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2222.2222222222222</c:v>
+                  <c:v>2064.7058823529414</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2361.1111111111109</c:v>
+                  <c:v>2182.3529411764707</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2500</c:v>
+                  <c:v>2300</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1253,7 +1273,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-8E52-4609-B15F-ADFD5A2DC54B}"/>
+              <c16:uniqueId val="{00000008-AEB0-4BDA-973B-92593FC7D8B6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1265,11 +1285,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="840848368"/>
-        <c:axId val="1204218144"/>
+        <c:axId val="1235898223"/>
+        <c:axId val="1235885743"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="840848368"/>
+        <c:axId val="1235898223"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1315,7 +1335,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1382,12 +1401,12 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1204218144"/>
+        <c:crossAx val="1235885743"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1204218144"/>
+        <c:axId val="1235885743"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1433,7 +1452,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1500,7 +1518,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="840848368"/>
+        <c:crossAx val="1235898223"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1514,7 +1532,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1546,7 +1563,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1554,6 +1570,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2705,22 +2722,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>19051</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>160233</xdr:rowOff>
+      <xdr:colOff>54428</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>179615</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>243797</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>82550</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>604157</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>8081</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Рисунок 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0C594D2-1765-873C-ED0B-6EBF3D86663F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E12711B-0F7F-4AB3-833D-DD8D91B7D0A5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2728,15 +2745,16 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
+      <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect b="54402"/>
-        <a:stretch/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="628651" y="528533"/>
-          <a:ext cx="7539946" cy="1027217"/>
+          <a:off x="707571" y="364672"/>
+          <a:ext cx="549729" cy="753752"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2747,23 +2765,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>102816</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>92528</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>10886</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>488950</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>141513</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>113311</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Рисунок 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{970F2F7E-4D1E-E098-2B94-C20AD6B8AF56}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0966392-8A5F-8C6F-7404-A8EA48209D25}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2779,8 +2797,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="609600" y="2128466"/>
-          <a:ext cx="8413750" cy="1503734"/>
+          <a:off x="3946071" y="10886"/>
+          <a:ext cx="1355271" cy="287482"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2791,23 +2809,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>598178</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>304799</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>32659</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>53975</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>468085</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>150954</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Рисунок 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{771582BE-A8CE-B67E-ACD7-33D5A4694C1B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44B7B3EF-8D9B-4480-0EC7-17F4216123A2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2823,8 +2841,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="598178" y="3917950"/>
-          <a:ext cx="8990322" cy="1476375"/>
+          <a:off x="6117770" y="32659"/>
+          <a:ext cx="1469572" cy="303352"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2833,131 +2851,25 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>469900</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>636815</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>38101</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>450850</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="6" name="Прямая со стрелкой 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B99FDE8D-DA69-AEDD-5BA9-9922BB56B09D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1" flipV="1">
-          <a:off x="10223500" y="793750"/>
-          <a:ext cx="1200150" cy="3073400"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent2"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent2"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent2"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>469900</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="7" name="Прямая со стрелкой 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E40E2E42-4822-599F-A456-9D3197D57B64}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1" flipV="1">
-          <a:off x="10223500" y="2311400"/>
-          <a:ext cx="996950" cy="1816100"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent2"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent2"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent2"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>582612</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>128588</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>1779814</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>172358</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Рисунок 8">
+        <xdr:cNvPr id="5" name="Рисунок 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3785C88-4F24-3EE2-CFD7-2B61A2F5195A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA0E754B-8CAF-EE75-004C-4C8B3406D291}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2973,8 +2885,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="582612" y="5746750"/>
-          <a:ext cx="9299576" cy="1282700"/>
+          <a:off x="8409215" y="38101"/>
+          <a:ext cx="1796142" cy="319314"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>6223</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>12441</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>492881</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>155510</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Рисунок 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47B8161D-C651-E1AB-55F6-A9B3E3BAD6F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="659366" y="4491135"/>
+          <a:ext cx="486658" cy="889518"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2985,59 +2941,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>139960</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>178836</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>139958</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>178838</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="10" name="Диаграмма 9">
+        <xdr:cNvPr id="7" name="Диаграмма 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82DD5F45-F26B-8AA4-0466-206FDFFDB1E9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="11" name="Диаграмма 10">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{678B0230-B283-F0DD-795D-73D6E246363F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4D1DDC0B-9788-5751-82C0-201EE5EA045E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3057,285 +2977,397 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>146050</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>186612</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:rowOff>163285</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>186613</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>163287</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="Прямоугольник 11">
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Диаграмма 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EFE65844-6655-AD55-15BA-6100918D2478}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FFA13159-5FA4-97B6-254B-0662F1BD984D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>272142</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>46652</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>178836</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>54429</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Рисунок 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E5AB2D3-84F9-2341-F03A-7FD70290C742}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="146050" y="336550"/>
-          <a:ext cx="425450" cy="527050"/>
+          <a:off x="8047652" y="4525346"/>
+          <a:ext cx="559837" cy="1127450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
       </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="ru-RU" sz="2400">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>1</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>120650</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>77755</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>124408</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>546100</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>23327</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>178837</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="Прямоугольник 12">
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="11" name="Прямая со стрелкой 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BF86174-DCD7-0058-4857-2FAF7E8E7C3D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0540D006-EFDE-2EA6-72C1-324F94507D05}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="120650" y="2044700"/>
-          <a:ext cx="425450" cy="527050"/>
+        <a:xfrm flipH="1">
+          <a:off x="3281265" y="4976327"/>
+          <a:ext cx="3864429" cy="1360714"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="straightConnector1">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent4"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="ru-RU" sz="2400">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>2</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>107950</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>38878</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>645368</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>147735</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="Прямоугольник 13">
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="12" name="Прямая со стрелкой 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33117034-50DF-8FAA-AC17-7D53F54F9E42}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C4A7EE13-822A-1B2E-7FCD-5D857712BA65}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="107950" y="3784600"/>
-          <a:ext cx="425450" cy="527050"/>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="3242388" y="3172408"/>
+          <a:ext cx="3872204" cy="2013857"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="straightConnector1">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent4"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="ru-RU" sz="2400">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>3</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>404325</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>178837</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>520700</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>163285</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>38878</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="Прямоугольник 14">
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="17" name="Прямая со стрелкой 16">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F070F645-E345-BE79-A90D-6A01F6A79EDF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E4B54EC-7270-71B8-7751-7E4B07DEE380}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="95250" y="5638800"/>
-          <a:ext cx="425450" cy="527050"/>
+        <a:xfrm flipH="1">
+          <a:off x="2923591" y="552061"/>
+          <a:ext cx="2402633" cy="3965511"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="straightConnector1">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent4"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
       </xdr:spPr>
       <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:fillRef>
         <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
+          <a:scrgbClr r="0" g="0" b="0"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="ru-RU" sz="2400">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>4</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>520957</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>155511</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>69980</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>54429</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="19" name="Прямая со стрелкой 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{077F9D19-F83F-54AF-A2A0-48C3AAC7C019}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="3040223" y="528735"/>
+          <a:ext cx="4152124" cy="4191000"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent4"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>54428</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>85530</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>15550</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>46652</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="21" name="Прямая со стрелкой 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CCF2A2C-33AA-D23D-3C9C-4137FD66BF84}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="3257938" y="2884714"/>
+          <a:ext cx="7550021" cy="2013857"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="accent4"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+          <a:round/>
+          <a:headEnd type="none" w="med" len="med"/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Info"/>
     </sheetNames>
     <definedNames>
       <definedName name="encode_feed"/>
-      <definedName name="encode_pipe"/>
-      <definedName name="encode_pipe_construction"/>
+      <definedName name="encode_json"/>
+      <definedName name="encode_pipe_diam"/>
+      <definedName name="encode_pipe_object"/>
+      <definedName name="encode_pipe_trajectory"/>
       <definedName name="encode_PVT"/>
       <definedName name="encode_t_model"/>
       <definedName name="MF_pipe_p_atma"/>
@@ -3358,39 +3390,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Стандартная">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -3442,7 +3474,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -3553,13 +3585,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -3568,6 +3593,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -3632,1018 +3664,1116 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F928C9B4-96B0-44FC-A159-E31844A45A17}">
   <sheetPr codeName="Лист1"/>
-  <dimension ref="B1:Y66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="C3:Q57"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="3" max="3" width="17.15234375" customWidth="1"/>
+    <col min="4" max="4" width="9.61328125" customWidth="1"/>
+    <col min="13" max="13" width="33.3828125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+    <row r="3" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="3" t="str">
+        <f>[1]!encode_pipe_trajectory(G6:H9)</f>
+        <v>{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,1900,2300]}</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="3" t="str">
+        <f>[1]!encode_pipe_diam(J6:K9,K4)</f>
+        <v>{"diam_list_mm":{"hmes_m":[0,500,2100],"diam_int_mm":[62,72,125]},"roughness_m":0.0001}</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.86</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="1"/>
+      <c r="J4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1E-4</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="M5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2">
+        <v>120</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N6" s="2">
+        <v>2.4251999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2">
+        <v>130</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1000</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1000</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2">
+        <v>62</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N7" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="8" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2">
+        <v>80</v>
+      </c>
+      <c r="G8" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1900</v>
+      </c>
+      <c r="J8" s="2">
+        <v>500</v>
+      </c>
+      <c r="K8" s="2">
+        <v>72</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="2">
+        <v>6.9649999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2500</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2300</v>
+      </c>
+      <c r="J9" s="2">
+        <v>2100</v>
+      </c>
+      <c r="K9" s="2">
+        <v>125</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N9" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="M10" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="N10" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0</v>
+      </c>
+      <c r="M11" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q4" s="3" t="str">
-        <f>[1]!encode_pipe_construction(P7:Q10,R7:S10)</f>
-        <v>{"h_list_m":{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,2000,2500]},"diam_list_mm":{"hmes_m":[0,500,2100,2500],"diam_int_mm":[62,62,125,125]}}</v>
-      </c>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-    </row>
-    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P5" s="1" t="s">
+      <c r="N11" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="3" t="str">
+        <f>[1]!encode_PVT(D3,D4,D5,D6,D7,D8,D9,D10,D11)</f>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0}</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2">
+        <v>30</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N13" s="2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C14" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2">
+        <v>10</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N14" s="2">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2">
+        <v>120</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="N15" s="5" t="str">
+        <f>[1]!encode_json(M6:N14)</f>
+        <v>{"thermal_conductivity_formation_WmC":2.4252,"specific_heat_capacity_formation_JkgC":200,"thermal_conductivity_cement_WmC":6.965,"thermal_conductivity_tubing_WmC":32,"thermal_conductivity_casing_WmC":32,"heat_transfer_casing_liquid_Wm2C":200,"heat_transfer_casing_gas_Wm2C":10,"heat_transfer_fluid_convection_Wm2C ":200,"time_calc_hr":240}</v>
+      </c>
+    </row>
+    <row r="16" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2">
         <v>0</v>
       </c>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1" t="s">
+      <c r="M16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N16" s="3" t="str">
+        <f>[1]!encode_t_model(N3,M19:N22,N4,N5,N15)</f>
+        <v>{"t_model":1,"t_list_C":{"hvert_m":[0,1000,2000,2500],"t_C":[10,35,80,90]}}</v>
+      </c>
+    </row>
+    <row r="17" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3" t="str">
+        <f>[1]!encode_feed(D13,D14,D15,D16,D12)</f>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":30,"fw_perc":10,"rp_m3m3":120}</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N17" s="1"/>
+    </row>
+    <row r="18" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="M18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="M19" s="2">
+        <v>0</v>
+      </c>
+      <c r="N19" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="M20" s="2">
+        <v>1000</v>
+      </c>
+      <c r="N20" s="2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="G21" s="4"/>
+      <c r="M21" s="2">
+        <v>2000</v>
+      </c>
+      <c r="N21" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="M22" s="2">
+        <v>2500</v>
+      </c>
+      <c r="N22" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C25" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="5" t="str">
+        <f>pipe_trajectory</f>
+        <v>{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,1900,2300]}</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K25" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C26" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="5" t="str">
+        <f>pipe_diam</f>
+        <v>{"diam_list_mm":{"hmes_m":[0,500,2100],"diam_int_mm":[62,72,125]},"roughness_m":0.0001}</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K26" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C27" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" s="5" t="str">
+        <f>t_model</f>
+        <v>{"t_model":1,"t_list_C":{"hvert_m":[0,1000,2000,2500],"t_C":[10,35,80,90]}}</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K27" s="5" t="str">
+        <f>pipe_object</f>
+        <v>{"construction":{"h_list_m":{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,1900,2300]},"diam_list_mm":{"hmes_m":[0,500,2100],"diam_int_mm":[62,72,125]},"roughness_m":0.0001},"t_model":{"t_model":1,"t_list_C":{"hvert_m":[0,1000,2000,2500],"t_C":[10,35,80,90]}},"flow_correlation":0,"flow_along_coord":false,"calibr_grav":1,"calibr_fric":1,"h_start_m":0,"h_end_m":0,"znlf":false}</v>
+      </c>
+    </row>
+    <row r="28" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C28" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K28" s="5" t="str">
+        <f>feed_json</f>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":30,"fw_perc":10,"rp_m3m3":120}</v>
+      </c>
+    </row>
+    <row r="29" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="2">
+        <v>0</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="K29" s="2">
         <v>1</v>
       </c>
-      <c r="S5" s="1"/>
-    </row>
-    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P7" s="2">
+    </row>
+    <row r="30" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C30" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D30" s="2">
+        <v>1</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C31" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K31" s="2"/>
+    </row>
+    <row r="32" spans="3:14" x14ac:dyDescent="0.4">
+      <c r="C32" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" s="2"/>
+      <c r="J32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K32" s="2"/>
+    </row>
+    <row r="33" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="C33" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="J33" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K33" s="2"/>
+    </row>
+    <row r="34" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="C34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="J34" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K34" s="2"/>
+    </row>
+    <row r="35" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="C35" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D35" s="3" t="str">
+        <f>[1]!encode_pipe_object(D25,D26,D27,D28,D29,D30,D31,D32,D33,D34)</f>
+        <v>{"construction":{"h_list_m":{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,1900,2300]},"diam_list_mm":{"hmes_m":[0,500,2100],"diam_int_mm":[62,72,125]},"roughness_m":0.0001},"t_model":{"t_model":1,"t_list_C":{"hvert_m":[0,1000,2000,2500],"t_C":[10,35,80,90]}},"flow_correlation":0,"flow_along_coord":false,"calibr_grav":1,"calibr_fric":1,"h_start_m":0,"h_end_m":0,"znlf":false}</v>
+      </c>
+      <c r="J35" s="6">
+        <f t="array" ref="J35:Q57">[1]!MF_pipe_p_atma(K25, K26, K27, K28, K29, K30, K31, K32, K33, K34)</f>
+        <v>207.53399999999999</v>
+      </c>
+      <c r="K35" s="6">
+        <v>25</v>
+      </c>
+      <c r="L35" s="6">
+        <v>10</v>
+      </c>
+      <c r="M35" s="6">
+        <v>207.53399999999999</v>
+      </c>
+      <c r="N35" s="6">
+        <v>86</v>
+      </c>
+      <c r="O35" s="6">
+        <v>1</v>
+      </c>
+      <c r="P35" s="6">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="6" t="str">
+        <v>["set show_log=1 in param to show calc log"]</v>
+      </c>
+    </row>
+    <row r="36" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J36" s="6" t="str">
+        <v>p_result_atma</v>
+      </c>
+      <c r="K36" s="6" t="str">
+        <v>p_1, atma</v>
+      </c>
+      <c r="L36" s="6" t="str">
+        <v>t_1, C</v>
+      </c>
+      <c r="M36" s="6" t="str">
+        <v>p_2, atma</v>
+      </c>
+      <c r="N36" s="6" t="str">
+        <v>t_2, C</v>
+      </c>
+      <c r="O36" s="6" t="str">
+        <v>calibr_grav</v>
+      </c>
+      <c r="P36" s="6" t="str">
+        <v>calibr_fric</v>
+      </c>
+      <c r="Q36" s="6" t="str">
+        <v>log</v>
+      </c>
+    </row>
+    <row r="37" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J37" s="6" t="str">
+        <v>h,m</v>
+      </c>
+      <c r="K37" s="6" t="str">
+        <v>hvert,m</v>
+      </c>
+      <c r="L37" s="6" t="str">
+        <v>p,atma</v>
+      </c>
+      <c r="M37" s="6" t="str">
+        <v>t,C</v>
+      </c>
+      <c r="N37" s="6" t="str">
+        <v>t_amb, C</v>
+      </c>
+      <c r="O37" s="6" t="str">
+        <v>Hl, %</v>
+      </c>
+      <c r="P37" s="6" t="str">
+        <v>fpat</v>
+      </c>
+      <c r="Q37" s="6" t="str">
+        <v>diam, mm</v>
+      </c>
+    </row>
+    <row r="38" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J38" s="6">
         <v>0</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="K38" s="6">
         <v>0</v>
       </c>
-      <c r="R7" s="4">
+      <c r="L38" s="6">
+        <v>25</v>
+      </c>
+      <c r="M38" s="6">
+        <v>10</v>
+      </c>
+      <c r="N38" s="6">
+        <v>10</v>
+      </c>
+      <c r="O38" s="6">
+        <v>100</v>
+      </c>
+      <c r="P38" s="6">
         <v>0</v>
       </c>
-      <c r="S7" s="4">
+      <c r="Q38" s="6">
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P8" s="2">
-        <v>1000</v>
-      </c>
-      <c r="Q8" s="2">
-        <v>1000</v>
-      </c>
-      <c r="R8" s="4">
+    <row r="39" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J39" s="6">
+        <v>147.05882352941177</v>
+      </c>
+      <c r="K39" s="6">
+        <v>147.05882352941177</v>
+      </c>
+      <c r="L39" s="6">
+        <v>37.211265919476702</v>
+      </c>
+      <c r="M39" s="6">
+        <v>13.676470588235293</v>
+      </c>
+      <c r="N39" s="6">
+        <v>13.676470588235293</v>
+      </c>
+      <c r="O39" s="6">
+        <v>100</v>
+      </c>
+      <c r="P39" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="6">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J40" s="6">
+        <v>294.11764705882354</v>
+      </c>
+      <c r="K40" s="6">
+        <v>294.11764705882354</v>
+      </c>
+      <c r="L40" s="6">
+        <v>49.336935976810224</v>
+      </c>
+      <c r="M40" s="6">
+        <v>17.352941176470587</v>
+      </c>
+      <c r="N40" s="6">
+        <v>17.352941176470587</v>
+      </c>
+      <c r="O40" s="6">
+        <v>100</v>
+      </c>
+      <c r="P40" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="6">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="41" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J41" s="6">
+        <v>441.1764705882353</v>
+      </c>
+      <c r="K41" s="6">
+        <v>441.1764705882353</v>
+      </c>
+      <c r="L41" s="6">
+        <v>61.368662604850357</v>
+      </c>
+      <c r="M41" s="6">
+        <v>21.029411764705884</v>
+      </c>
+      <c r="N41" s="6">
+        <v>21.029411764705884</v>
+      </c>
+      <c r="O41" s="6">
+        <v>100</v>
+      </c>
+      <c r="P41" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="6">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J42" s="6">
         <v>500</v>
       </c>
-      <c r="S8" s="4">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P9" s="2">
-        <v>2000</v>
-      </c>
-      <c r="Q9" s="2">
-        <v>2000</v>
-      </c>
-      <c r="R9" s="4">
+      <c r="K42" s="6">
+        <v>500</v>
+      </c>
+      <c r="L42" s="6">
+        <v>66.154734668379703</v>
+      </c>
+      <c r="M42" s="6">
+        <v>22.5</v>
+      </c>
+      <c r="N42" s="6">
+        <v>22.5</v>
+      </c>
+      <c r="O42" s="6">
+        <v>100</v>
+      </c>
+      <c r="P42" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="43" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J43" s="6">
+        <v>588.23529411764707</v>
+      </c>
+      <c r="K43" s="6">
+        <v>588.23529411764707</v>
+      </c>
+      <c r="L43" s="6">
+        <v>73.301276031794316</v>
+      </c>
+      <c r="M43" s="6">
+        <v>24.705882352941178</v>
+      </c>
+      <c r="N43" s="6">
+        <v>24.705882352941178</v>
+      </c>
+      <c r="O43" s="6">
+        <v>100</v>
+      </c>
+      <c r="P43" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="44" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J44" s="6">
+        <v>735.29411764705878</v>
+      </c>
+      <c r="K44" s="6">
+        <v>735.29411764705878</v>
+      </c>
+      <c r="L44" s="6">
+        <v>85.131937480979204</v>
+      </c>
+      <c r="M44" s="6">
+        <v>28.382352941176471</v>
+      </c>
+      <c r="N44" s="6">
+        <v>28.382352941176471</v>
+      </c>
+      <c r="O44" s="6">
+        <v>100</v>
+      </c>
+      <c r="P44" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="45" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J45" s="6">
+        <v>882.35294117647061</v>
+      </c>
+      <c r="K45" s="6">
+        <v>882.35294117647061</v>
+      </c>
+      <c r="L45" s="6">
+        <v>96.859528861433972</v>
+      </c>
+      <c r="M45" s="6">
+        <v>32.058823529411768</v>
+      </c>
+      <c r="N45" s="6">
+        <v>32.058823529411768</v>
+      </c>
+      <c r="O45" s="6">
+        <v>100</v>
+      </c>
+      <c r="P45" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="46" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J46" s="6">
+        <v>1029.4117647058824</v>
+      </c>
+      <c r="K46" s="6">
+        <v>1026.4705882352941</v>
+      </c>
+      <c r="L46" s="6">
+        <v>108.25265963744981</v>
+      </c>
+      <c r="M46" s="6">
+        <v>36.191176470588239</v>
+      </c>
+      <c r="N46" s="6">
+        <v>36.191176470588239</v>
+      </c>
+      <c r="O46" s="6">
+        <v>100</v>
+      </c>
+      <c r="P46" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="47" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J47" s="6">
+        <v>1176.4705882352941</v>
+      </c>
+      <c r="K47" s="6">
+        <v>1158.8235294117646</v>
+      </c>
+      <c r="L47" s="6">
+        <v>118.64374732377269</v>
+      </c>
+      <c r="M47" s="6">
+        <v>42.147058823529413</v>
+      </c>
+      <c r="N47" s="6">
+        <v>42.147058823529413</v>
+      </c>
+      <c r="O47" s="6">
+        <v>100</v>
+      </c>
+      <c r="P47" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="48" spans="3:17" x14ac:dyDescent="0.4">
+      <c r="J48" s="6">
+        <v>1323.5294117647059</v>
+      </c>
+      <c r="K48" s="6">
+        <v>1291.1764705882354</v>
+      </c>
+      <c r="L48" s="6">
+        <v>129.01643292775486</v>
+      </c>
+      <c r="M48" s="6">
+        <v>48.102941176470587</v>
+      </c>
+      <c r="N48" s="6">
+        <v>48.102941176470587</v>
+      </c>
+      <c r="O48" s="6">
+        <v>100</v>
+      </c>
+      <c r="P48" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="49" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J49" s="6">
+        <v>1470.5882352941176</v>
+      </c>
+      <c r="K49" s="6">
+        <v>1423.5294117647059</v>
+      </c>
+      <c r="L49" s="6">
+        <v>139.37296783267652</v>
+      </c>
+      <c r="M49" s="6">
+        <v>54.058823529411761</v>
+      </c>
+      <c r="N49" s="6">
+        <v>54.058823529411761</v>
+      </c>
+      <c r="O49" s="6">
+        <v>100</v>
+      </c>
+      <c r="P49" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="50" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J50" s="6">
+        <v>1617.6470588235295</v>
+      </c>
+      <c r="K50" s="6">
+        <v>1555.8823529411766</v>
+      </c>
+      <c r="L50" s="6">
+        <v>149.71212069474134</v>
+      </c>
+      <c r="M50" s="6">
+        <v>60.014705882352942</v>
+      </c>
+      <c r="N50" s="6">
+        <v>60.014705882352942</v>
+      </c>
+      <c r="O50" s="6">
+        <v>100</v>
+      </c>
+      <c r="P50" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="51" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J51" s="6">
+        <v>1764.7058823529412</v>
+      </c>
+      <c r="K51" s="6">
+        <v>1688.2352941176471</v>
+      </c>
+      <c r="L51" s="6">
+        <v>160.03289583994723</v>
+      </c>
+      <c r="M51" s="6">
+        <v>65.970588235294116</v>
+      </c>
+      <c r="N51" s="6">
+        <v>65.970588235294116</v>
+      </c>
+      <c r="O51" s="6">
+        <v>100</v>
+      </c>
+      <c r="P51" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="52" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J52" s="6">
+        <v>1911.7647058823529</v>
+      </c>
+      <c r="K52" s="6">
+        <v>1820.5882352941176</v>
+      </c>
+      <c r="L52" s="6">
+        <v>170.33447407582048</v>
+      </c>
+      <c r="M52" s="6">
+        <v>71.92647058823529</v>
+      </c>
+      <c r="N52" s="6">
+        <v>71.92647058823529</v>
+      </c>
+      <c r="O52" s="6">
+        <v>100</v>
+      </c>
+      <c r="P52" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="53" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J53" s="6">
+        <v>2058.8235294117649</v>
+      </c>
+      <c r="K53" s="6">
+        <v>1947.0588235294119</v>
+      </c>
+      <c r="L53" s="6">
+        <v>180.15967523685279</v>
+      </c>
+      <c r="M53" s="6">
+        <v>77.617647058823536</v>
+      </c>
+      <c r="N53" s="6">
+        <v>77.617647058823536</v>
+      </c>
+      <c r="O53" s="6">
+        <v>100</v>
+      </c>
+      <c r="P53" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="6">
+        <v>72.000000000000014</v>
+      </c>
+    </row>
+    <row r="54" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J54" s="6">
         <v>2100</v>
       </c>
-      <c r="S9" s="4">
+      <c r="K54" s="6">
+        <v>1980</v>
+      </c>
+      <c r="L54" s="6">
+        <v>182.71586855800516</v>
+      </c>
+      <c r="M54" s="6">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="N54" s="6">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="O54" s="6">
+        <v>100</v>
+      </c>
+      <c r="P54" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="6">
         <v>125</v>
       </c>
     </row>
-    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P10" s="2">
+    <row r="55" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J55" s="6">
+        <v>2205.8823529411766</v>
+      </c>
+      <c r="K55" s="6">
+        <v>2064.7058823529414</v>
+      </c>
+      <c r="L55" s="6">
+        <v>189.28532313169057</v>
+      </c>
+      <c r="M55" s="6">
+        <v>81.294117647058826</v>
+      </c>
+      <c r="N55" s="6">
+        <v>81.294117647058826</v>
+      </c>
+      <c r="O55" s="6">
+        <v>100</v>
+      </c>
+      <c r="P55" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="56" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J56" s="6">
+        <v>2352.9411764705883</v>
+      </c>
+      <c r="K56" s="6">
+        <v>2182.3529411764707</v>
+      </c>
+      <c r="L56" s="6">
+        <v>198.40957045644666</v>
+      </c>
+      <c r="M56" s="6">
+        <v>83.647058823529406</v>
+      </c>
+      <c r="N56" s="6">
+        <v>83.647058823529406</v>
+      </c>
+      <c r="O56" s="6">
+        <v>100</v>
+      </c>
+      <c r="P56" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="57" spans="10:17" x14ac:dyDescent="0.4">
+      <c r="J57" s="6">
         <v>2500</v>
       </c>
-      <c r="Q10" s="2">
-        <v>2500</v>
-      </c>
-      <c r="R10" s="4"/>
-      <c r="S10" s="4"/>
-    </row>
-    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q13" s="3" t="str">
-        <f>[1]!encode_t_model(1,P16:Q19)</f>
-        <v>{"t_model":1,"t_list_C":{"hvert_m":[0,2500],"t_C":[10,58]}}</v>
-      </c>
-    </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="Q14" s="1"/>
-    </row>
-    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P16" s="2">
+      <c r="K57" s="6">
+        <v>2300</v>
+      </c>
+      <c r="L57" s="6">
+        <v>207.53360232980467</v>
+      </c>
+      <c r="M57" s="6">
+        <v>86</v>
+      </c>
+      <c r="N57" s="6">
+        <v>86</v>
+      </c>
+      <c r="O57" s="6">
+        <v>100</v>
+      </c>
+      <c r="P57" s="6">
         <v>0</v>
       </c>
-      <c r="Q16" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P17" s="2">
-        <v>2500</v>
-      </c>
-      <c r="Q17" s="2">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-    </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-    </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="S22" s="5" t="str">
-        <f>pipe_construction</f>
-        <v>{"h_list_m":{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,2000,2500]},"diam_list_mm":{"hmes_m":[0,500,2100,2500],"diam_int_mm":[62,62,125,125]}}</v>
-      </c>
-    </row>
-    <row r="23" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R23" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="S23" s="5" t="str">
-        <f>t_model</f>
-        <v>{"t_model":1,"t_list_C":{"hvert_m":[0,2500],"t_C":[10,58]}}</v>
-      </c>
-    </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="S24" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R25" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="S25" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R26" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="S26" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R27" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="S27" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R28" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="S28" s="2"/>
-    </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R29" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S29" s="2"/>
-    </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="R30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S30" s="2"/>
-    </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>33</v>
-      </c>
-      <c r="R31" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S31" s="3" t="str">
-        <f>[1]!encode_pipe(S22,S23,S24,S25,S26,S27,S28,S29,S30)</f>
-        <v>{"construction":{"h_list_m":{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,2000,2500]},"diam_list_mm":{"hmes_m":[0,500,2100,2500],"diam_int_mm":[62,62,125,125]}},"t_model":{"t_model":1,"t_list_C":{"hvert_m":[0,2500],"t_C":[10,58]}},"flow_correlation":0,"flow_along_coord":false,"calibr_grav":1,"calibr_fric":1,"h_start_m":0,"h_end_m":0,"znlf":false}</v>
-      </c>
-    </row>
-    <row r="34" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R34" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="S34" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R35" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="S35" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="36" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R36" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="S36" s="5" t="str">
-        <f>pipe_object</f>
-        <v>{"construction":{"h_list_m":{"hmes_m":[0,1000,2000,2500],"hvert_m":[0,1000,2000,2500]},"diam_list_mm":{"hmes_m":[0,500,2100,2500],"diam_int_mm":[62,62,125,125]}},"t_model":{"t_model":1,"t_list_C":{"hvert_m":[0,2500],"t_C":[10,58]}},"flow_correlation":0,"flow_along_coord":false,"calibr_grav":1,"calibr_fric":1,"h_start_m":0,"h_end_m":0,"znlf":false}</v>
-      </c>
-    </row>
-    <row r="37" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R37" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="S37" s="5" t="str">
-        <f>feed_json</f>
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":50,"fw_perc":100,"rp_m3m3":120}</v>
-      </c>
-    </row>
-    <row r="38" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R38" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S38" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R39" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="S39" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="40" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R40" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="S40" s="2"/>
-    </row>
-    <row r="41" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R41" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="S41" s="2"/>
-    </row>
-    <row r="42" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R42" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="S42" s="2"/>
-    </row>
-    <row r="43" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R43" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="S43" s="2"/>
-    </row>
-    <row r="44" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H44" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I44" s="2">
-        <v>0.6</v>
-      </c>
-      <c r="R44" s="6">
-        <f t="array" ref="R44:Y66">[1]!MF_pipe_p_atma(S34, S35, S36, S37, S38, S39, S40, S41, S42, S43)</f>
-        <v>275.262</v>
-      </c>
-      <c r="S44" s="6">
-        <v>10</v>
-      </c>
-      <c r="T44" s="6">
-        <v>10</v>
-      </c>
-      <c r="U44" s="6">
-        <v>275.262</v>
-      </c>
-      <c r="V44" s="6">
-        <v>58</v>
-      </c>
-      <c r="W44" s="6">
-        <v>1</v>
-      </c>
-      <c r="X44" s="6">
-        <v>1</v>
-      </c>
-      <c r="Y44" s="6" t="str">
-        <v>["set show_log=1 in param to show calc log"]</v>
-      </c>
-    </row>
-    <row r="45" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H45" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I45" s="2">
-        <v>0.86</v>
-      </c>
-      <c r="R45" s="6" t="str">
-        <v>p_result_atma</v>
-      </c>
-      <c r="S45" s="6" t="str">
-        <v>p_1, atma</v>
-      </c>
-      <c r="T45" s="6" t="str">
-        <v>t_1, C</v>
-      </c>
-      <c r="U45" s="6" t="str">
-        <v>p_2, atma</v>
-      </c>
-      <c r="V45" s="6" t="str">
-        <v>t_2, C</v>
-      </c>
-      <c r="W45" s="6" t="str">
-        <v>calibr_grav</v>
-      </c>
-      <c r="X45" s="6" t="str">
-        <v>calibr_fric</v>
-      </c>
-      <c r="Y45" s="6" t="str">
-        <v>log</v>
-      </c>
-    </row>
-    <row r="46" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H46" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="I46" s="2">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="R46" s="6" t="str">
-        <v>h,m</v>
-      </c>
-      <c r="S46" s="6" t="str">
-        <v>hvert,m</v>
-      </c>
-      <c r="T46" s="6" t="str">
-        <v>p,atma</v>
-      </c>
-      <c r="U46" s="6" t="str">
-        <v>t,C</v>
-      </c>
-      <c r="V46" s="6" t="str">
-        <v>t_amb, C</v>
-      </c>
-      <c r="W46" s="6" t="str">
-        <v>Hl, %</v>
-      </c>
-      <c r="X46" s="6" t="str">
-        <v>fpat</v>
-      </c>
-      <c r="Y46" s="6" t="str">
-        <v>diam, mm</v>
-      </c>
-    </row>
-    <row r="47" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H47" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I47" s="2">
-        <v>120</v>
-      </c>
-      <c r="R47" s="6">
-        <v>0</v>
-      </c>
-      <c r="S47" s="6">
-        <v>0</v>
-      </c>
-      <c r="T47" s="6">
-        <v>10</v>
-      </c>
-      <c r="U47" s="6">
-        <v>10</v>
-      </c>
-      <c r="V47" s="6">
-        <v>10</v>
-      </c>
-      <c r="W47" s="6">
-        <v>100</v>
-      </c>
-      <c r="X47" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y47" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="48" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H48" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I48" s="2">
-        <v>130</v>
-      </c>
-      <c r="R48" s="6">
-        <v>138.88888888888889</v>
-      </c>
-      <c r="S48" s="6">
-        <v>138.88888888888889</v>
-      </c>
-      <c r="T48" s="6">
-        <v>24.836360057558057</v>
-      </c>
-      <c r="U48" s="6">
-        <v>12.666666666666666</v>
-      </c>
-      <c r="V48" s="6">
-        <v>12.666666666666666</v>
-      </c>
-      <c r="W48" s="6">
-        <v>100</v>
-      </c>
-      <c r="X48" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y48" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="49" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H49" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I49" s="2">
-        <v>80</v>
-      </c>
-      <c r="R49" s="6">
-        <v>277.77777777777777</v>
-      </c>
-      <c r="S49" s="6">
-        <v>277.77777777777777</v>
-      </c>
-      <c r="T49" s="6">
-        <v>39.660912169855287</v>
-      </c>
-      <c r="U49" s="6">
-        <v>15.333333333333334</v>
-      </c>
-      <c r="V49" s="6">
-        <v>15.333333333333334</v>
-      </c>
-      <c r="W49" s="6">
-        <v>100</v>
-      </c>
-      <c r="X49" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y49" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="50" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H50" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I50" s="2">
-        <v>1.2</v>
-      </c>
-      <c r="R50" s="6">
-        <v>416.66666666666663</v>
-      </c>
-      <c r="S50" s="6">
-        <v>416.66666666666663</v>
-      </c>
-      <c r="T50" s="6">
-        <v>54.473728023011631</v>
-      </c>
-      <c r="U50" s="6">
-        <v>18</v>
-      </c>
-      <c r="V50" s="6">
-        <v>18</v>
-      </c>
-      <c r="W50" s="6">
-        <v>100</v>
-      </c>
-      <c r="X50" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y50" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="51" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H51" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I51" s="2">
-        <v>0.6</v>
-      </c>
-      <c r="R51" s="6">
-        <v>555.55555555555554</v>
-      </c>
-      <c r="S51" s="6">
-        <v>555.55555555555554</v>
-      </c>
-      <c r="T51" s="6">
-        <v>69.274877304399666</v>
-      </c>
-      <c r="U51" s="6">
-        <v>20.666666666666664</v>
-      </c>
-      <c r="V51" s="6">
-        <v>20.666666666666664</v>
-      </c>
-      <c r="W51" s="6">
-        <v>100</v>
-      </c>
-      <c r="X51" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y51" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="52" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H52" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="I52" s="2">
-        <v>0</v>
-      </c>
-      <c r="R52" s="6">
-        <v>694.44444444444446</v>
-      </c>
-      <c r="S52" s="6">
-        <v>694.44444444444446</v>
-      </c>
-      <c r="T52" s="6">
-        <v>84.064262054326051</v>
-      </c>
-      <c r="U52" s="6">
-        <v>23.333333333333332</v>
-      </c>
-      <c r="V52" s="6">
-        <v>23.333333333333332</v>
-      </c>
-      <c r="W52" s="6">
-        <v>100</v>
-      </c>
-      <c r="X52" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y52" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="53" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H53" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="I53" s="3" t="str">
-        <f>[1]!encode_PVT(I44,I45,I46,I47,I48,I49,I50,I51,I52)</f>
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0}</v>
-      </c>
-      <c r="R53" s="6">
-        <v>833.33333333333326</v>
-      </c>
-      <c r="S53" s="6">
-        <v>833.33333333333326</v>
-      </c>
-      <c r="T53" s="6">
-        <v>98.841955005012849</v>
-      </c>
-      <c r="U53" s="6">
-        <v>26</v>
-      </c>
-      <c r="V53" s="6">
-        <v>26</v>
-      </c>
-      <c r="W53" s="6">
-        <v>100</v>
-      </c>
-      <c r="X53" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y53" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="54" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H54" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I54" s="2">
-        <v>50</v>
-      </c>
-      <c r="R54" s="6">
-        <v>972.22222222222217</v>
-      </c>
-      <c r="S54" s="6">
-        <v>972.22222222222217</v>
-      </c>
-      <c r="T54" s="6">
-        <v>113.60819486374973</v>
-      </c>
-      <c r="U54" s="6">
-        <v>28.666666666666664</v>
-      </c>
-      <c r="V54" s="6">
-        <v>28.666666666666664</v>
-      </c>
-      <c r="W54" s="6">
-        <v>100</v>
-      </c>
-      <c r="X54" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y54" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="55" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H55" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I55" s="2">
-        <v>100</v>
-      </c>
-      <c r="R55" s="6">
-        <v>1111.1111111111111</v>
-      </c>
-      <c r="S55" s="6">
-        <v>1111.1111111111111</v>
-      </c>
-      <c r="T55" s="6">
-        <v>128.36305394047776</v>
-      </c>
-      <c r="U55" s="6">
-        <v>31.333333333333332</v>
-      </c>
-      <c r="V55" s="6">
-        <v>31.333333333333332</v>
-      </c>
-      <c r="W55" s="6">
-        <v>100</v>
-      </c>
-      <c r="X55" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y55" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="56" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H56" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I56" s="2">
-        <v>120</v>
-      </c>
-      <c r="R56" s="6">
-        <v>1250</v>
-      </c>
-      <c r="S56" s="6">
-        <v>1250</v>
-      </c>
-      <c r="T56" s="6">
-        <v>143.10660666796306</v>
-      </c>
-      <c r="U56" s="6">
-        <v>34</v>
-      </c>
-      <c r="V56" s="6">
-        <v>34</v>
-      </c>
-      <c r="W56" s="6">
-        <v>100</v>
-      </c>
-      <c r="X56" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y56" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="57" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H57" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I57" s="2">
-        <v>0</v>
-      </c>
-      <c r="R57" s="6">
-        <v>1388.8888888888889</v>
-      </c>
-      <c r="S57" s="6">
-        <v>1388.8888888888889</v>
-      </c>
-      <c r="T57" s="6">
-        <v>157.83860705561924</v>
-      </c>
-      <c r="U57" s="6">
-        <v>36.666666666666664</v>
-      </c>
-      <c r="V57" s="6">
-        <v>36.666666666666664</v>
-      </c>
-      <c r="W57" s="6">
-        <v>100</v>
-      </c>
-      <c r="X57" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y57" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="58" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="H58" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I58" s="3" t="str">
-        <f>[1]!encode_feed(I54,I55,I56,I57,I53)</f>
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":50,"fw_perc":100,"rp_m3m3":120}</v>
-      </c>
-      <c r="R58" s="6">
-        <v>1527.7777777777778</v>
-      </c>
-      <c r="S58" s="6">
-        <v>1527.7777777777778</v>
-      </c>
-      <c r="T58" s="6">
-        <v>172.55946291726846</v>
-      </c>
-      <c r="U58" s="6">
-        <v>39.333333333333329</v>
-      </c>
-      <c r="V58" s="6">
-        <v>39.333333333333329</v>
-      </c>
-      <c r="W58" s="6">
-        <v>100</v>
-      </c>
-      <c r="X58" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y58" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="59" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R59" s="6">
-        <v>1666.6666666666665</v>
-      </c>
-      <c r="S59" s="6">
-        <v>1666.6666666666665</v>
-      </c>
-      <c r="T59" s="6">
-        <v>187.26925720901431</v>
-      </c>
-      <c r="U59" s="6">
-        <v>41.999999999999993</v>
-      </c>
-      <c r="V59" s="6">
-        <v>41.999999999999993</v>
-      </c>
-      <c r="W59" s="6">
-        <v>100</v>
-      </c>
-      <c r="X59" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y59" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="60" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R60" s="6">
-        <v>1805.5555555555554</v>
-      </c>
-      <c r="S60" s="6">
-        <v>1805.5555555555554</v>
-      </c>
-      <c r="T60" s="6">
-        <v>201.96807608679808</v>
-      </c>
-      <c r="U60" s="6">
-        <v>44.666666666666657</v>
-      </c>
-      <c r="V60" s="6">
-        <v>44.666666666666657</v>
-      </c>
-      <c r="W60" s="6">
-        <v>100</v>
-      </c>
-      <c r="X60" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y60" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="61" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R61" s="6">
-        <v>1944.4444444444443</v>
-      </c>
-      <c r="S61" s="6">
-        <v>1944.4444444444443</v>
-      </c>
-      <c r="T61" s="6">
-        <v>216.65585276159905</v>
-      </c>
-      <c r="U61" s="6">
-        <v>47.333333333333329</v>
-      </c>
-      <c r="V61" s="6">
-        <v>47.333333333333329</v>
-      </c>
-      <c r="W61" s="6">
-        <v>100</v>
-      </c>
-      <c r="X61" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y61" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="62" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R62" s="6">
-        <v>2083.3333333333335</v>
-      </c>
-      <c r="S62" s="6">
-        <v>2083.3333333333335</v>
-      </c>
-      <c r="T62" s="6">
-        <v>231.33268489206455</v>
-      </c>
-      <c r="U62" s="6">
-        <v>50</v>
-      </c>
-      <c r="V62" s="6">
-        <v>50</v>
-      </c>
-      <c r="W62" s="6">
-        <v>100</v>
-      </c>
-      <c r="X62" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y62" s="6">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="63" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R63" s="6">
-        <v>2100</v>
-      </c>
-      <c r="S63" s="6">
-        <v>2100</v>
-      </c>
-      <c r="T63" s="6">
-        <v>233.09334496046432</v>
-      </c>
-      <c r="U63" s="6">
-        <v>50.319999999999993</v>
-      </c>
-      <c r="V63" s="6">
-        <v>50.319999999999993</v>
-      </c>
-      <c r="W63" s="6">
-        <v>100</v>
-      </c>
-      <c r="X63" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y63" s="6">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="64" spans="8:25" x14ac:dyDescent="0.25">
-      <c r="R64" s="6">
-        <v>2222.2222222222222</v>
-      </c>
-      <c r="S64" s="6">
-        <v>2222.2222222222222</v>
-      </c>
-      <c r="T64" s="6">
-        <v>245.98725456824823</v>
-      </c>
-      <c r="U64" s="6">
-        <v>52.666666666666664</v>
-      </c>
-      <c r="V64" s="6">
-        <v>52.666666666666664</v>
-      </c>
-      <c r="W64" s="6">
-        <v>100</v>
-      </c>
-      <c r="X64" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y64" s="6">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="65" spans="18:25" x14ac:dyDescent="0.25">
-      <c r="R65" s="6">
-        <v>2361.1111111111109</v>
-      </c>
-      <c r="S65" s="6">
-        <v>2361.1111111111109</v>
-      </c>
-      <c r="T65" s="6">
-        <v>260.62969555631469</v>
-      </c>
-      <c r="U65" s="6">
-        <v>55.333333333333329</v>
-      </c>
-      <c r="V65" s="6">
-        <v>55.333333333333329</v>
-      </c>
-      <c r="W65" s="6">
-        <v>100</v>
-      </c>
-      <c r="X65" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y65" s="6">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="66" spans="18:25" x14ac:dyDescent="0.25">
-      <c r="R66" s="6">
-        <v>2500</v>
-      </c>
-      <c r="S66" s="6">
-        <v>2500</v>
-      </c>
-      <c r="T66" s="6">
-        <v>275.2616896761848</v>
-      </c>
-      <c r="U66" s="6">
-        <v>57.999999999999993</v>
-      </c>
-      <c r="V66" s="6">
-        <v>57.999999999999993</v>
-      </c>
-      <c r="W66" s="6">
-        <v>100</v>
-      </c>
-      <c r="X66" s="6">
-        <v>3</v>
-      </c>
-      <c r="Y66" s="6">
+      <c r="Q57" s="6">
         <v>125</v>
       </c>
     </row>

</xml_diff>